<commit_message>
removed extra sheet in menumanager
</commit_message>
<xml_diff>
--- a/menuManager.xlsx
+++ b/menuManager.xlsx
@@ -20,7 +20,6 @@
     <sheet name="stat" sheetId="3" r:id="rId5"/>
     <sheet name="input" sheetId="1" r:id="rId6"/>
     <sheet name="code" sheetId="10" r:id="rId7"/>
-    <sheet name="makes" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028" calcCompleted="0"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="330" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="160">
   <si>
     <t>sample</t>
   </si>
@@ -521,114 +520,6 @@
   </si>
   <si>
     <t>cits_fixed_nocovariate_esadj</t>
-  </si>
-  <si>
-    <t>parm</t>
-  </si>
-  <si>
-    <t>es</t>
-  </si>
-  <si>
-    <t>c1</t>
-  </si>
-  <si>
-    <t>c2</t>
-  </si>
-  <si>
-    <t>make_with</t>
-  </si>
-  <si>
-    <t>mtotal</t>
-  </si>
-  <si>
-    <t>result$mt+result$mc</t>
-  </si>
-  <si>
-    <t>Pm</t>
-  </si>
-  <si>
-    <t>result$mt/(result$mt+result$mc)</t>
-  </si>
-  <si>
-    <t>Proportion of blocks in treatment</t>
-  </si>
-  <si>
-    <t>Proportion of clusters in treatment</t>
-  </si>
-  <si>
-    <t>Proportion of longitudinal units in treatment</t>
-  </si>
-  <si>
-    <t>mbar</t>
-  </si>
-  <si>
-    <t>2/(1/result$mt+1/result$mc)</t>
-  </si>
-  <si>
-    <t>Harmonic mean of blocks</t>
-  </si>
-  <si>
-    <t>Harmonic mean of clusters</t>
-  </si>
-  <si>
-    <t>Harmonic mean of longitudinal units</t>
-  </si>
-  <si>
-    <t>ntotal</t>
-  </si>
-  <si>
-    <t>result$nt+result$nc</t>
-  </si>
-  <si>
-    <t>Pn</t>
-  </si>
-  <si>
-    <t>result$nt/(result$nt+result$nc)</t>
-  </si>
-  <si>
-    <t>Proportion of individuals in treatment</t>
-  </si>
-  <si>
-    <t>nbar</t>
-  </si>
-  <si>
-    <t>2/(1/result$nt+1/result$nc)</t>
-  </si>
-  <si>
-    <t>Harmonic mean of individuals in blocks</t>
-  </si>
-  <si>
-    <t>Harmonic mean of individuals in clusters</t>
-  </si>
-  <si>
-    <t>Harmonic mean of individuals in longitudinal units</t>
-  </si>
-  <si>
-    <t>totaltime</t>
-  </si>
-  <si>
-    <t>result$pretime+result$posttime</t>
-  </si>
-  <si>
-    <t>Number timepoints</t>
-  </si>
-  <si>
-    <t>Ptime</t>
-  </si>
-  <si>
-    <t>result$posttime/(result$pretime+result$posttime)</t>
-  </si>
-  <si>
-    <t>Proportion of timepoints after treatment</t>
-  </si>
-  <si>
-    <t>iccbar</t>
-  </si>
-  <si>
-    <t>1-result$icc</t>
-  </si>
-  <si>
-    <t>1-ICC</t>
   </si>
 </sst>
 </file>
@@ -2625,514 +2516,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CFF29F0-411E-4DB5-B08C-646123839D2C}">
-  <dimension ref="A1:AK16"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="2.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="2.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="45.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="23" max="24" width="46.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:37" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:37" s="1" customFormat="1">
-      <c r="A2" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2"/>
-      <c r="G2"/>
-      <c r="H2"/>
-      <c r="I2"/>
-      <c r="J2"/>
-      <c r="K2"/>
-      <c r="L2"/>
-      <c r="M2"/>
-      <c r="N2"/>
-      <c r="O2"/>
-      <c r="P2"/>
-      <c r="Q2"/>
-      <c r="R2"/>
-      <c r="S2"/>
-      <c r="T2" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="X2" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" s="1" customFormat="1">
-      <c r="A3" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3"/>
-      <c r="G3"/>
-      <c r="H3"/>
-      <c r="I3"/>
-      <c r="J3"/>
-      <c r="K3"/>
-      <c r="L3"/>
-      <c r="M3"/>
-      <c r="N3"/>
-      <c r="O3"/>
-      <c r="P3"/>
-      <c r="Q3"/>
-      <c r="R3"/>
-      <c r="S3"/>
-      <c r="T3" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="U3" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="V3" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="W3" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="X3" s="1" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37" s="1" customFormat="1">
-      <c r="A4" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4" t="b">
-        <v>1</v>
-      </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4"/>
-      <c r="G4"/>
-      <c r="H4"/>
-      <c r="I4"/>
-      <c r="J4"/>
-      <c r="K4"/>
-      <c r="L4"/>
-      <c r="M4"/>
-      <c r="N4"/>
-      <c r="O4"/>
-      <c r="P4"/>
-      <c r="Q4"/>
-      <c r="R4"/>
-      <c r="S4"/>
-      <c r="T4" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="W4" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="X4" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:37" s="1" customFormat="1">
-      <c r="A5" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="B5"/>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="E5"/>
-      <c r="F5"/>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5"/>
-      <c r="J5"/>
-      <c r="K5"/>
-      <c r="L5"/>
-      <c r="M5"/>
-      <c r="N5"/>
-      <c r="O5"/>
-      <c r="P5"/>
-      <c r="Q5"/>
-      <c r="R5"/>
-      <c r="S5"/>
-      <c r="T5" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="W5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="X5" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:37" s="1" customFormat="1">
-      <c r="A6" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="B6"/>
-      <c r="C6"/>
-      <c r="D6"/>
-      <c r="E6"/>
-      <c r="F6"/>
-      <c r="G6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6"/>
-      <c r="J6"/>
-      <c r="K6"/>
-      <c r="L6"/>
-      <c r="M6"/>
-      <c r="N6"/>
-      <c r="O6"/>
-      <c r="P6"/>
-      <c r="Q6"/>
-      <c r="R6"/>
-      <c r="S6"/>
-      <c r="T6" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="W6" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="X6" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="7" spans="1:37" s="1" customFormat="1">
-      <c r="A7" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B7"/>
-      <c r="C7"/>
-      <c r="D7"/>
-      <c r="E7"/>
-      <c r="F7"/>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7"/>
-      <c r="J7"/>
-      <c r="K7"/>
-      <c r="L7"/>
-      <c r="M7"/>
-      <c r="N7"/>
-      <c r="O7"/>
-      <c r="P7"/>
-      <c r="Q7"/>
-      <c r="R7"/>
-      <c r="S7"/>
-      <c r="T7" s="1" t="s">
-        <v>183</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="W7" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="X7" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="8" spans="1:37" s="1" customFormat="1">
-      <c r="A8" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="B8"/>
-      <c r="C8"/>
-      <c r="D8"/>
-      <c r="E8"/>
-      <c r="F8"/>
-      <c r="G8"/>
-      <c r="H8"/>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" t="b">
-        <v>1</v>
-      </c>
-      <c r="K8"/>
-      <c r="L8"/>
-      <c r="M8"/>
-      <c r="N8"/>
-      <c r="O8"/>
-      <c r="P8"/>
-      <c r="Q8"/>
-      <c r="R8"/>
-      <c r="S8"/>
-      <c r="T8" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="W8" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="X8" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="9" spans="1:37" s="1" customFormat="1">
-      <c r="A9" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="B9"/>
-      <c r="C9"/>
-      <c r="D9"/>
-      <c r="E9"/>
-      <c r="F9"/>
-      <c r="G9"/>
-      <c r="H9"/>
-      <c r="I9" t="b">
-        <v>1</v>
-      </c>
-      <c r="J9" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9"/>
-      <c r="L9"/>
-      <c r="M9"/>
-      <c r="N9"/>
-      <c r="O9"/>
-      <c r="P9"/>
-      <c r="Q9"/>
-      <c r="R9"/>
-      <c r="S9"/>
-      <c r="T9" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="W9" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="X9" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:37" s="1" customFormat="1">
-      <c r="A10" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B10"/>
-      <c r="C10"/>
-      <c r="D10"/>
-      <c r="E10"/>
-      <c r="F10"/>
-      <c r="G10"/>
-      <c r="H10"/>
-      <c r="I10"/>
-      <c r="J10"/>
-      <c r="K10" t="b">
-        <v>1</v>
-      </c>
-      <c r="L10"/>
-      <c r="M10"/>
-      <c r="N10"/>
-      <c r="O10"/>
-      <c r="P10"/>
-      <c r="Q10"/>
-      <c r="R10"/>
-      <c r="S10"/>
-      <c r="T10" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="W10" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="X10" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="13" spans="1:37">
-      <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
-      <c r="V13" s="1"/>
-      <c r="W13" s="1"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="1"/>
-      <c r="Z13" s="1"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="1"/>
-      <c r="AC13" s="1"/>
-      <c r="AD13" s="1"/>
-      <c r="AE13" s="1"/>
-      <c r="AF13" s="1"/>
-      <c r="AG13" s="1"/>
-      <c r="AH13" s="1"/>
-      <c r="AI13" s="1"/>
-      <c r="AJ13" s="1"/>
-      <c r="AK13" s="1"/>
-    </row>
-    <row r="16" spans="1:37">
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fixed too small a sample with covar, still need to tweak
</commit_message>
<xml_diff>
--- a/menuManager.xlsx
+++ b/menuManager.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10509"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hedbergec/Dropbox/Papers/Papers.QEDs/Apps/plannerApp/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6749A151-8273-F245-BF27-EF731CD39086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38673797-AC6D-C346-B23F-EA31C717FC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2200" yWindow="2200" windowWidth="21480" windowHeight="14540" firstSheet="6" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="2200" yWindow="2200" windowWidth="21480" windowHeight="14540" firstSheet="5" activeTab="5" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="sample" sheetId="5" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <sheet name="input" sheetId="1" r:id="rId6"/>
     <sheet name="code" sheetId="10" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="191028" calcCompleted="0"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -318,9 +318,6 @@
     <t>q</t>
   </si>
   <si>
-    <t>c(0,20)</t>
-  </si>
-  <si>
     <t>Number covariates</t>
   </si>
   <si>
@@ -520,13 +517,16 @@
   </si>
   <si>
     <t>cits_fixed_nocovariate_esadj</t>
+  </si>
+  <si>
+    <t>c(0,6)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -883,9 +883,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -893,7 +893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -901,7 +901,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -917,12 +917,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -936,7 +936,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -947,7 +947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -958,7 +958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -969,7 +969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -980,7 +980,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -999,13 +999,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.140625" customWidth="1"/>
+    <col min="3" max="3" width="5.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1028,7 +1028,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1048,7 +1048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1070,14 +1070,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -1123,7 +1123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1148,13 +1148,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="99.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="99.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -1200,7 +1200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -1223,7 +1223,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1269,27 +1269,27 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7085B87C-0BDF-4509-A80F-252767BE3B26}">
   <dimension ref="A1:W16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="5.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="7.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="7.85546875" style="1" customWidth="1"/>
-    <col min="14" max="14" width="5.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="9.140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="49.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="55.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="9.140625" style="1"/>
+    <col min="10" max="10" width="9.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="7.83203125" style="1" customWidth="1"/>
+    <col min="14" max="14" width="5.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="9.1640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="21" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="55.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="24" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>36</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>46</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>1</v>
       </c>
       <c r="O2" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P2" s="1">
         <v>100</v>
@@ -1416,7 +1416,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>51</v>
       </c>
@@ -1472,7 +1472,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>55</v>
       </c>
@@ -1528,7 +1528,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>59</v>
       </c>
@@ -1557,7 +1557,7 @@
         <v>1</v>
       </c>
       <c r="O5" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P5" s="1">
         <v>100</v>
@@ -1581,7 +1581,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>63</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>68</v>
       </c>
@@ -1699,7 +1699,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>73</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>75</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>77</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>80</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="12" spans="1:23">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>84</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>88</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>91</v>
       </c>
@@ -2049,33 +2049,33 @@
         <v>0</v>
       </c>
       <c r="P14" s="1">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="Q14" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="R14" s="1">
+        <v>1</v>
+      </c>
+      <c r="S14" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="R14" s="1">
-        <v>1</v>
-      </c>
-      <c r="S14" s="1" t="s">
+      <c r="T14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="U14" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="V14" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="W14" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23">
-      <c r="A15" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -2102,21 +2102,21 @@
         <v>0.2</v>
       </c>
       <c r="T15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="U15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="V15" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="W15" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="U15" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="V15" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="W15" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23">
-      <c r="A16" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -2140,22 +2140,22 @@
         <v>3</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="R16" s="1">
         <v>0.15</v>
       </c>
       <c r="T16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="U16" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="U16" s="1" t="s">
+      <c r="V16" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="V16" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="W16" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2167,350 +2167,350 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
   <dimension ref="A1:D47"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.95">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.95">
-      <c r="A2" s="2" t="s">
+      <c r="B2" t="s">
         <v>102</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.95">
-      <c r="A3" s="2" t="s">
+      <c r="B3" t="s">
         <v>104</v>
       </c>
-      <c r="B3" t="s">
+    </row>
+    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.95">
-      <c r="A4" s="2" t="s">
+      <c r="B4" t="s">
         <v>106</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>107</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.95">
-      <c r="A5" s="2" t="s">
+      <c r="B5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.95">
-      <c r="A6" s="2" t="s">
+      <c r="B6" t="s">
         <v>110</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.95">
-      <c r="A7" s="2" t="s">
+      <c r="B7" t="s">
+        <v>106</v>
+      </c>
+      <c r="C7" t="s">
         <v>112</v>
       </c>
-      <c r="B7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C7" t="s">
+    </row>
+    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="15.95">
-      <c r="A8" s="2" t="s">
+      <c r="B8" t="s">
         <v>114</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.95">
-      <c r="A9" s="2" t="s">
+      <c r="B9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C9" t="s">
         <v>116</v>
       </c>
-      <c r="B9" t="s">
-        <v>115</v>
-      </c>
-      <c r="C9" t="s">
+    </row>
+    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="15.95">
-      <c r="A10" s="2" t="s">
+      <c r="B10" t="s">
         <v>118</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>119</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>120</v>
       </c>
-      <c r="D10" t="s">
+    </row>
+    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.95">
-      <c r="A11" s="2" t="s">
+      <c r="B11" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B11" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.95">
-      <c r="A12" s="2" t="s">
+      <c r="B12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C12" t="s">
         <v>123</v>
       </c>
-      <c r="B12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.95">
-      <c r="A13" s="2" t="s">
+      <c r="B13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D13" t="s">
         <v>125</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B15" t="s">
         <v>119</v>
       </c>
-      <c r="C13" t="s">
-        <v>120</v>
-      </c>
-      <c r="D13" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.95">
-      <c r="A14" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B14" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.95">
-      <c r="A15" s="2" t="s">
+      <c r="C15" t="s">
         <v>128</v>
       </c>
-      <c r="B15" t="s">
-        <v>120</v>
-      </c>
-      <c r="C15" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.95">
-      <c r="A16" s="2" t="s">
+      <c r="B16" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" t="s">
         <v>130</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" t="s">
         <v>119</v>
       </c>
-      <c r="C16" t="s">
-        <v>120</v>
-      </c>
-      <c r="D16" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.95">
-      <c r="A17" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B17" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15.95">
-      <c r="A18" s="2" t="s">
+      <c r="C18" t="s">
         <v>133</v>
       </c>
-      <c r="B18" t="s">
-        <v>120</v>
-      </c>
-      <c r="C18" t="s">
+    </row>
+    <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="15.95">
-      <c r="A19" s="2" t="s">
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" t="s">
+        <v>119</v>
+      </c>
+      <c r="D19" t="s">
         <v>135</v>
       </c>
-      <c r="B19" t="s">
-        <v>119</v>
-      </c>
-      <c r="C19" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" t="s">
+    </row>
+    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="15.95">
-      <c r="A20" s="2" t="s">
+      <c r="B20" t="s">
         <v>137</v>
       </c>
-      <c r="B20" t="s">
+    </row>
+    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.95">
-      <c r="A21" s="2" t="s">
+      <c r="B21" t="s">
         <v>139</v>
       </c>
-      <c r="B21" t="s">
+    </row>
+    <row r="22" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.95">
-      <c r="A22" s="2" t="s">
+      <c r="B22" t="s">
         <v>141</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>142</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>143</v>
       </c>
-      <c r="D22" t="s">
+    </row>
+    <row r="23" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.95">
-      <c r="A23" s="2" t="s">
+      <c r="B23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B23" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.95">
-      <c r="A24" s="2" t="s">
+      <c r="B24" t="s">
         <v>146</v>
       </c>
-      <c r="B24" t="s">
+    </row>
+    <row r="25" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="15.95">
-      <c r="A25" s="2" t="s">
+      <c r="B25" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" t="s">
         <v>148</v>
       </c>
-      <c r="B25" t="s">
-        <v>142</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.95">
-      <c r="A26" s="2" t="s">
+      <c r="B26" t="s">
         <v>150</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.95">
-      <c r="A27" s="2" t="s">
+    <row r="28" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.95">
-      <c r="A28" s="2" t="s">
+    <row r="29" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15.95">
-      <c r="A29" s="2" t="s">
+    <row r="30" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" ht="15.95">
-      <c r="A30" s="2" t="s">
+      <c r="B30" t="s">
         <v>155</v>
       </c>
-      <c r="B30" t="s">
+    </row>
+    <row r="31" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15.95">
-      <c r="A31" s="2" t="s">
+    <row r="32" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="2" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="15.95">
-      <c r="A32" s="2" t="s">
+    <row r="33" spans="1:1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="2" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="15.95">
-      <c r="A33" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="15.95">
+    <row r="34" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
     </row>
-    <row r="35" spans="1:1" ht="15.95">
+    <row r="35" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
     </row>
-    <row r="36" spans="1:1" ht="15.95">
+    <row r="36" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
     </row>
-    <row r="37" spans="1:1" ht="15.95">
+    <row r="37" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
     </row>
-    <row r="38" spans="1:1" ht="15.95">
+    <row r="38" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
     </row>
-    <row r="39" spans="1:1" ht="15.95">
+    <row r="39" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
     </row>
-    <row r="40" spans="1:1" ht="15.95">
+    <row r="40" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
     </row>
-    <row r="41" spans="1:1" ht="15.95">
+    <row r="41" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
     </row>
-    <row r="42" spans="1:1" ht="15.95">
+    <row r="42" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
     </row>
-    <row r="43" spans="1:1" ht="15.95">
+    <row r="43" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
     </row>
-    <row r="44" spans="1:1" ht="15.95">
+    <row r="44" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
     </row>
-    <row r="45" spans="1:1" ht="15.95">
+    <row r="45" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
     </row>
-    <row r="46" spans="1:1" ht="15.95">
+    <row r="46" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
     </row>
-    <row r="47" spans="1:1" ht="15.95">
+    <row r="47" spans="1:1" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add m-distance, new labels from excel from beth
</commit_message>
<xml_diff>
--- a/menuManager.xlsx
+++ b/menuManager.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hedbe\Dropbox\Papers\Paper.QEDs\Apps\plannerApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACCEB44-AD76-4CB1-B745-26CAA602F590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D7EA79D-AB9A-4D58-883A-C6113842A624}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2940" windowWidth="16875" windowHeight="10643" tabRatio="716" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
+    <workbookView xWindow="3615" yWindow="3615" windowWidth="16875" windowHeight="10643" tabRatio="716" activeTab="6" xr2:uid="{8D89E9AD-B3C8-4CE6-A909-5B9DBA95DCBB}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="11" r:id="rId1"/>
@@ -149,7 +149,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="169">
   <si>
     <t>sample</t>
   </si>
@@ -175,33 +175,18 @@
     <t>srs</t>
   </si>
   <si>
-    <t>Simple random sample</t>
-  </si>
-  <si>
     <t>blocked</t>
   </si>
   <si>
-    <t>Blocked treatments</t>
-  </si>
-  <si>
     <t>clustered</t>
   </si>
   <si>
-    <t>Clustered treatments</t>
-  </si>
-  <si>
     <t>its</t>
   </si>
   <si>
-    <t>Interrupted time series</t>
-  </si>
-  <si>
     <t>cits</t>
   </si>
   <si>
-    <t>Comparative interrupted time series</t>
-  </si>
-  <si>
     <t>inference</t>
   </si>
   <si>
@@ -223,15 +208,9 @@
     <t>nocovariate</t>
   </si>
   <si>
-    <t>Without controls</t>
-  </si>
-  <si>
     <t>covariate</t>
   </si>
   <si>
-    <t>With controls</t>
-  </si>
-  <si>
     <t>stat</t>
   </si>
   <si>
@@ -286,120 +265,36 @@
     <t>m</t>
   </si>
   <si>
-    <t>Number blocks</t>
-  </si>
-  <si>
-    <t>Number clusters</t>
-  </si>
-  <si>
-    <t>Number longitudinal units</t>
-  </si>
-  <si>
     <t>mt</t>
   </si>
   <si>
-    <t>Treatment number blocks</t>
-  </si>
-  <si>
-    <t>Treatment number clusters</t>
-  </si>
-  <si>
-    <t>Treatment number longitudinal units</t>
-  </si>
-  <si>
     <t>mc</t>
   </si>
   <si>
-    <t>Comparison number blocks</t>
-  </si>
-  <si>
-    <t>Comparison number clusters</t>
-  </si>
-  <si>
-    <t>Comparison number longitudinal units</t>
-  </si>
-  <si>
     <t>n</t>
   </si>
   <si>
-    <t>Number individuals in blocks</t>
-  </si>
-  <si>
-    <t>Number individuals in clusters</t>
-  </si>
-  <si>
-    <t>Number individuals in longitudinal units</t>
-  </si>
-  <si>
     <t>nt</t>
   </si>
   <si>
-    <t>Treatment number of individuals</t>
-  </si>
-  <si>
-    <t>Treatment number of individuals in blocks</t>
-  </si>
-  <si>
-    <t>Treatment number of individuals in clusters</t>
-  </si>
-  <si>
-    <t>Treatment number of individuals in longitudinal units</t>
-  </si>
-  <si>
     <t>nc</t>
   </si>
   <si>
-    <t>Comparison number of individuals</t>
-  </si>
-  <si>
-    <t>Comparison number of individuals in blocks</t>
-  </si>
-  <si>
-    <t>Comparison number of individuals in clusters</t>
-  </si>
-  <si>
-    <t>Comparison number of individuals in longitudinal units</t>
-  </si>
-  <si>
     <t>pretime</t>
   </si>
   <si>
-    <t>Number timepoints before treatment</t>
-  </si>
-  <si>
     <t>posttime</t>
   </si>
   <si>
-    <t>Number timepoints after treatment</t>
-  </si>
-  <si>
     <t>icc</t>
   </si>
   <si>
-    <t>intraclass correlation</t>
-  </si>
-  <si>
     <t>R2_1</t>
   </si>
   <si>
-    <t>Outcome variance reduction in outcome</t>
-  </si>
-  <si>
-    <t>Outcome variance reduction in outcome (individuals)</t>
-  </si>
-  <si>
     <t>R2_2</t>
   </si>
   <si>
-    <t>Outcome variance reduction in outcome (blocks)</t>
-  </si>
-  <si>
-    <t>Outcome variance reduction in outcome (clusters)</t>
-  </si>
-  <si>
-    <t>Outcome variance reduction in outcome (longitudinal units)</t>
-  </si>
-  <si>
     <t>ar</t>
   </si>
   <si>
@@ -598,9 +493,6 @@
     <t>did</t>
   </si>
   <si>
-    <t>Difference in Difference</t>
-  </si>
-  <si>
     <t>label_did</t>
   </si>
   <si>
@@ -650,13 +542,127 @@
   </si>
   <si>
     <t>&lt;- This sheet notes which designs, inference, model, etc., need which elements for stats</t>
+  </si>
+  <si>
+    <t>Blocked Random Assignment</t>
+  </si>
+  <si>
+    <t>Clustered Random Assignment</t>
+  </si>
+  <si>
+    <t>Simple Random Assignment</t>
+  </si>
+  <si>
+    <t>Without covariates</t>
+  </si>
+  <si>
+    <t>With covariates</t>
+  </si>
+  <si>
+    <t>Number of interention group  longitudinal units</t>
+  </si>
+  <si>
+    <t>Number of comparison group longitudinal units</t>
+  </si>
+  <si>
+    <t>Number of intervention group  individuals</t>
+  </si>
+  <si>
+    <t>Number of comparison group individuals</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (due to covariates)</t>
+  </si>
+  <si>
+    <t>Number of blocks</t>
+  </si>
+  <si>
+    <t>Number of intervention group blocks</t>
+  </si>
+  <si>
+    <t>Number of comparison group blocks</t>
+  </si>
+  <si>
+    <t>Intraclass correlation (ICC)</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (individuals)</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (blocks)</t>
+  </si>
+  <si>
+    <t>Number of  clusters</t>
+  </si>
+  <si>
+    <t>Number of intervention group clusters</t>
+  </si>
+  <si>
+    <t>Number of comparison  group clusters</t>
+  </si>
+  <si>
+    <t>Number individuals per  cluster</t>
+  </si>
+  <si>
+    <t>Number individuals per  block</t>
+  </si>
+  <si>
+    <t>Number of comparison  group individuals per  block</t>
+  </si>
+  <si>
+    <t>Number of intervention group individuals per block</t>
+  </si>
+  <si>
+    <t>Number of intervention group individuals per cluster</t>
+  </si>
+  <si>
+    <t>Number of comparison  group individuals per cluster</t>
+  </si>
+  <si>
+    <t>Number of timepoints before intervention</t>
+  </si>
+  <si>
+    <t>Number of timepoints after intervention</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (clusters)</t>
+  </si>
+  <si>
+    <t>Variance reduction in outcome (longitudinal units)</t>
+  </si>
+  <si>
+    <t>Number of covariates</t>
+  </si>
+  <si>
+    <t>Number of  longitudinal units</t>
+  </si>
+  <si>
+    <t>Number individuals per  longitudinal unit</t>
+  </si>
+  <si>
+    <t>Number of intervention group individuals per longitudinal unit</t>
+  </si>
+  <si>
+    <t>Number of comparison group  individuals per longitudinal unit</t>
+  </si>
+  <si>
+    <t>Number of intervention group individuals</t>
+  </si>
+  <si>
+    <t>Interrupted Time Series (ITS)</t>
+  </si>
+  <si>
+    <t>Comparative Interrupted Time Series (CITS)</t>
+  </si>
+  <si>
+    <t>Difference in Differences (DiD)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -675,6 +681,13 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -701,13 +714,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1070,19 +1086,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C51C3392-495A-4716-B7D0-8CB1570246E2}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>156</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -1091,7 +1107,7 @@
         <v>sample</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -1100,7 +1116,7 @@
         <v>design</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -1109,7 +1125,7 @@
         <v>inference</v>
       </c>
       <c r="B5" t="s">
-        <v>159</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -1118,7 +1134,7 @@
         <v>model</v>
       </c>
       <c r="B6" t="s">
-        <v>160</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -1127,7 +1143,7 @@
         <v>stat</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -1136,13 +1152,13 @@
         <v>input</v>
       </c>
       <c r="B8" t="s">
-        <v>166</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="3"/>
       <c r="C9" t="s">
-        <v>163</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -1151,12 +1167,12 @@
         <v>code</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>164</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -1167,7 +1183,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A96E0447-8401-42C5-BE02-401F505AE938}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
@@ -1201,9 +1217,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62AA0D0E-E4D1-469A-AF1F-085E17D5518F}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="29.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -1225,7 +1241,7 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1233,10 +1249,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>131</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1244,10 +1260,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1255,10 +1271,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>166</v>
       </c>
       <c r="D5" t="b">
         <v>0</v>
@@ -1266,10 +1282,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>167</v>
       </c>
       <c r="D6" t="b">
         <v>0</v>
@@ -1277,10 +1293,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>149</v>
+        <v>168</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
@@ -1294,7 +1310,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33C6AD60-7AB8-4CAF-9726-0F1707E818DE}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.1328125" customWidth="1"/>
@@ -1302,7 +1318,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1311,27 +1327,27 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
-      </c>
       <c r="H1" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1351,10 +1367,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
@@ -1371,16 +1387,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F39838A5-C062-40CB-BD39-4466E5E1974A}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.1328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1389,27 +1405,27 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
-      </c>
       <c r="H1" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>134</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1432,10 +1448,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>135</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1455,7 +1471,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9306200-6D5D-404E-9AA4-2D83AC7E89FD}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
@@ -1463,7 +1479,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -1472,27 +1488,27 @@
         <v>7</v>
       </c>
       <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
-      </c>
       <c r="H1" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1515,10 +1531,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1541,10 +1557,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1579,98 +1595,98 @@
     <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" style="1" customWidth="1"/>
     <col min="3" max="3" width="8" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="5.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.3984375" style="1" customWidth="1"/>
-    <col min="8" max="9" width="7.86328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="5.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.33203125" style="1" customWidth="1"/>
+    <col min="8" max="9" width="7.796875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.1328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="14" width="7.86328125" style="1" customWidth="1"/>
+    <col min="12" max="14" width="7.796875" style="1" customWidth="1"/>
     <col min="15" max="16" width="9.1328125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.73046875" style="1" bestFit="1" customWidth="1"/>
-    <col min="19" max="21" width="49.265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="55.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="19" max="21" width="49.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="23" width="55.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="16384" width="9.1328125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="P1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="T1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="X1" s="1" t="s">
-        <v>150</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1" t="b">
         <v>1</v>
@@ -1713,21 +1729,21 @@
         <v>c(4,40)</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>45</v>
+        <v>141</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>46</v>
+        <v>147</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>47</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="D3" s="1" t="b">
         <v>1</v>
@@ -1770,21 +1786,21 @@
         <v>c(2,40)</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>49</v>
+        <v>142</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>50</v>
+        <v>148</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>51</v>
+        <v>136</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>51</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="D4" s="1" t="b">
         <v>1</v>
@@ -1827,21 +1843,21 @@
         <v>c(2,40)</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>53</v>
+        <v>143</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>54</v>
+        <v>149</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>55</v>
+        <v>137</v>
       </c>
       <c r="W4" s="1" t="s">
-        <v>55</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="D5" s="1" t="b">
         <v>1</v>
@@ -1881,21 +1897,21 @@
         <v>c(4,150)</v>
       </c>
       <c r="T5" s="1" t="s">
-        <v>57</v>
+        <v>151</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>58</v>
+        <v>150</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>59</v>
+        <v>162</v>
       </c>
       <c r="W5" s="1" t="s">
-        <v>59</v>
+        <v>162</v>
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="B6" s="1" t="b">
         <v>1</v>
@@ -1941,27 +1957,27 @@
         <v>c(2,150)</v>
       </c>
       <c r="S6" s="1" t="s">
-        <v>61</v>
+        <v>138</v>
       </c>
       <c r="T6" s="1" t="s">
-        <v>62</v>
+        <v>153</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>63</v>
+        <v>154</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>64</v>
+        <v>163</v>
       </c>
       <c r="W6" s="1" t="s">
-        <v>64</v>
+        <v>163</v>
       </c>
       <c r="X6" s="1" t="s">
-        <v>61</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="B7" s="1" t="b">
         <v>1</v>
@@ -2007,27 +2023,27 @@
         <v>c(2,150)</v>
       </c>
       <c r="S7" s="1" t="s">
-        <v>66</v>
+        <v>139</v>
       </c>
       <c r="T7" s="1" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>68</v>
+        <v>155</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>69</v>
+        <v>164</v>
       </c>
       <c r="W7" s="1" t="s">
-        <v>69</v>
+        <v>164</v>
       </c>
       <c r="X7" s="1" t="s">
-        <v>66</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="E8" s="1" t="b">
         <v>1</v>
@@ -2071,21 +2087,21 @@
         <v>c(2,100)</v>
       </c>
       <c r="T8" s="1" t="s">
-        <v>71</v>
+        <v>156</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>71</v>
+        <v>156</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>71</v>
+        <v>156</v>
       </c>
       <c r="W8" s="1" t="s">
-        <v>71</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>72</v>
+        <v>44</v>
       </c>
       <c r="E9" s="1" t="b">
         <v>1</v>
@@ -2129,21 +2145,21 @@
         <v>c(2,100)</v>
       </c>
       <c r="T9" s="1" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
       <c r="W9" s="1" t="s">
-        <v>73</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A10" s="1" t="s">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="b">
         <v>1</v>
@@ -2186,21 +2202,21 @@
         <v>c(0.01,0.2)</v>
       </c>
       <c r="T10" s="1" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
       <c r="W10" s="1" t="s">
-        <v>75</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A11" s="1" t="s">
-        <v>76</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="b">
         <v>1</v>
@@ -2237,24 +2253,24 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="S11" s="1" t="s">
-        <v>77</v>
+        <v>140</v>
       </c>
       <c r="T11" s="1" t="s">
-        <v>78</v>
+        <v>145</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>78</v>
+        <v>145</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>78</v>
+        <v>145</v>
       </c>
       <c r="W11" s="1" t="s">
-        <v>78</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A12" s="1" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="D12" s="1" t="b">
         <v>1</v>
@@ -2282,21 +2298,21 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="T12" s="1" t="s">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="V12" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="W12" s="1" t="s">
-        <v>82</v>
+        <v>158</v>
+      </c>
+      <c r="V12" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="W12" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>48</v>
       </c>
       <c r="E13" s="1" t="b">
         <v>1</v>
@@ -2336,24 +2352,24 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="T13" s="1" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="W13" s="1" t="s">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="X13" s="1" t="s">
-        <v>151</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A14" s="1" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="B14" s="1" t="b">
         <v>1</v>
@@ -2393,24 +2409,24 @@
         <v>c(0,6)</v>
       </c>
       <c r="S14" s="1" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="T14" s="1" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="U14" s="1" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="V14" s="1" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
       <c r="W14" s="1" t="s">
-        <v>86</v>
+        <v>160</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A15" s="1" t="s">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="C15" s="1" t="b">
         <v>1</v>
@@ -2438,21 +2454,21 @@
         <v>c(0,0.99)</v>
       </c>
       <c r="T15" s="1" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="U15" s="1" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="V15" s="1" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
       <c r="W15" s="1" t="s">
-        <v>88</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A16" s="1" t="s">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="C16" s="1" t="b">
         <v>1</v>
@@ -2473,26 +2489,26 @@
         <v>0</v>
       </c>
       <c r="P16" s="1">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="Q16" s="1">
         <v>0.15</v>
       </c>
       <c r="R16" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>c(0,3)</v>
+        <v>c(0,3.25)</v>
       </c>
       <c r="T16" s="1" t="s">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="U16" s="1" t="s">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="V16" s="1" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="W16" s="1" t="s">
-        <v>92</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -2505,316 +2521,316 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D24D9501-1928-C24A-A5F8-EF63F20DDAEF}">
   <dimension ref="A1:D44"/>
-  <sheetFormatPr defaultColWidth="11.3984375" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="11.33203125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="33.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.86328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A2" s="2" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="2" t="s">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>97</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="B4" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A5" s="2" t="s">
-        <v>101</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A6" s="2" t="s">
-        <v>102</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A7" s="2" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A8" s="2" t="s">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="B8" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A9" s="2" t="s">
-        <v>108</v>
+        <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="C9" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A10" s="2" t="s">
-        <v>110</v>
+        <v>75</v>
       </c>
       <c r="B10" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="C10" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D10" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A11" s="2" t="s">
-        <v>114</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A12" s="2" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A13" s="2" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="B13" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>118</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A14" s="2" t="s">
-        <v>119</v>
+        <v>84</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A15" s="2" t="s">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
-        <v>121</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A16" s="2" t="s">
-        <v>122</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="C16" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D16" t="s">
-        <v>123</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A17" s="2" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A18" s="2" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A19" s="2" t="s">
-        <v>127</v>
+        <v>92</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>128</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A20" s="2" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="B20" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A21" s="2" t="s">
-        <v>131</v>
+        <v>96</v>
       </c>
       <c r="B21" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A22" s="2" t="s">
-        <v>133</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="D22" t="s">
-        <v>136</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A23" s="2" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="B23" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A24" s="2" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="B24" t="s">
-        <v>139</v>
+        <v>104</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A25" s="2" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="B25" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="C25" t="s">
-        <v>141</v>
+        <v>106</v>
       </c>
       <c r="D25" t="s">
-        <v>136</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A26" s="2" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A27" s="2" t="s">
-        <v>143</v>
+        <v>108</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A28" s="2" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A29" s="2" t="s">
-        <v>145</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A30" s="2" t="s">
-        <v>146</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A31" s="2" t="s">
-        <v>147</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A32" s="2" t="s">
-        <v>152</v>
+        <v>116</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A33" s="2" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
-        <v>97</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A34" s="2" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="B34" t="s">
-        <v>155</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="15.75" x14ac:dyDescent="0.5">

</xml_diff>